<commit_message>
Version sans la dernière mise à jour d'Antoine de y'a 2 j
</commit_message>
<xml_diff>
--- a/FitQuest_GameDesign.xlsx
+++ b/FitQuest_GameDesign.xlsx
@@ -23,6 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Référence" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚔️ Dégâts Combat" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💥 Limites" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🌟 Invocations" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚙️ Règles Invocations" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="45">
+  <fonts count="52">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -284,8 +286,47 @@
       <color rgb="FFBFDBFE"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FDE68A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00A5B4FC"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00EEF2FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00EEF2FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00A5B4FC"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FBBF24"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="65">
+  <fills count="72">
     <fill>
       <patternFill/>
     </fill>
@@ -607,8 +648,44 @@
         <fgColor rgb="FFEF4444"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D0826"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003B82F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00110D30"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B5CF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F59E0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1A2E"/>
+        <bgColor rgb="001A1A2E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -716,11 +793,58 @@
         <color rgb="FF2D1B69"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="002D2150"/>
+      </left>
+      <right style="thin">
+        <color rgb="002D2150"/>
+      </right>
+      <top style="thin">
+        <color rgb="002D2150"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002D2150"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="002D2150"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002D2150"/>
+      </right>
+      <top style="thin">
+        <color rgb="002D2150"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002D2150"/>
+      </right>
+      <top style="thin">
+        <color rgb="002D2150"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002D2150"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="164">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1199,6 +1323,61 @@
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="65" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="67" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="69" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="70" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="65" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="68" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="66" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="71" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7682,6 +7861,1114 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="164" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="164" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="164" t="inlineStr">
+        <is>
+          <t>icon</t>
+        </is>
+      </c>
+      <c r="D1" s="164" t="inlineStr">
+        <is>
+          <t>rarity</t>
+        </is>
+      </c>
+      <c r="E1" s="164" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F1" s="164" t="inlineStr">
+        <is>
+          <t>effect_type</t>
+        </is>
+      </c>
+      <c r="G1" s="164" t="inlineStr">
+        <is>
+          <t>base_damage</t>
+        </is>
+      </c>
+      <c r="H1" s="164" t="inlineStr">
+        <is>
+          <t>hits</t>
+        </is>
+      </c>
+      <c r="I1" s="164" t="inlineStr">
+        <is>
+          <t>stat_scale_stat</t>
+        </is>
+      </c>
+      <c r="J1" s="164" t="inlineStr">
+        <is>
+          <t>stat_scale_mult</t>
+        </is>
+      </c>
+      <c r="K1" s="164" t="inlineStr">
+        <is>
+          <t>side_effect_type</t>
+        </is>
+      </c>
+      <c r="L1" s="164" t="inlineStr">
+        <is>
+          <t>side_effect_value</t>
+        </is>
+      </c>
+      <c r="M1" s="164" t="inlineStr">
+        <is>
+          <t>instakill_thresh</t>
+        </is>
+      </c>
+      <c r="N1" s="164" t="inlineStr">
+        <is>
+          <t>gauge_required</t>
+        </is>
+      </c>
+      <c r="O1" s="164" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="P1" s="164" t="inlineStr">
+        <is>
+          <t>flavor</t>
+        </is>
+      </c>
+      <c r="Q1" s="164" t="inlineStr">
+        <is>
+          <t>obtain</t>
+        </is>
+      </c>
+      <c r="R1" s="164" t="inlineStr">
+        <is>
+          <t>obtain_desc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="165" t="inlineStr">
+        <is>
+          <t>titan</t>
+        </is>
+      </c>
+      <c r="B2" s="166" t="inlineStr">
+        <is>
+          <t>Titan</t>
+        </is>
+      </c>
+      <c r="C2" s="167" t="inlineStr">
+        <is>
+          <t>🗿</t>
+        </is>
+      </c>
+      <c r="D2" s="168" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="E2" s="167" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F2" s="167" t="inlineStr">
+        <is>
+          <t>damage_force</t>
+        </is>
+      </c>
+      <c r="G2" s="167" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" s="167" t="n"/>
+      <c r="I2" s="167" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="J2" s="167" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K2" s="167" t="n"/>
+      <c r="L2" s="167" t="n"/>
+      <c r="M2" s="167" t="n"/>
+      <c r="N2" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="169" t="inlineStr">
+        <is>
+          <t>Le colosse de pierre écrase l'ennemi sous son poing de granite.</t>
+        </is>
+      </c>
+      <c r="P2" s="169" t="inlineStr">
+        <is>
+          <t>« La montagne ne fléchit pas. »</t>
+        </is>
+      </c>
+      <c r="Q2" s="167" t="inlineStr">
+        <is>
+          <t>drop:giant_boar</t>
+        </is>
+      </c>
+      <c r="R2" s="169" t="inlineStr">
+        <is>
+          <t>Drop rare du Sanglier Géant</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="170" t="inlineStr">
+        <is>
+          <t>shiva</t>
+        </is>
+      </c>
+      <c r="B3" s="171" t="inlineStr">
+        <is>
+          <t>Shiva</t>
+        </is>
+      </c>
+      <c r="C3" s="172" t="inlineStr">
+        <is>
+          <t>❄️</t>
+        </is>
+      </c>
+      <c r="D3" s="168" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="E3" s="172" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="F3" s="172" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G3" s="172" t="n">
+        <v>110</v>
+      </c>
+      <c r="H3" s="172" t="n"/>
+      <c r="I3" s="172" t="n"/>
+      <c r="J3" s="172" t="n"/>
+      <c r="K3" s="172" t="inlineStr">
+        <is>
+          <t>boss_weaken</t>
+        </is>
+      </c>
+      <c r="L3" s="172" t="inlineStr">
+        <is>
+          <t>turns:1,reduction:0.5</t>
+        </is>
+      </c>
+      <c r="M3" s="172" t="n"/>
+      <c r="N3" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="173" t="inlineStr">
+        <is>
+          <t>Blizzard paralysant — réduit l'attaque du boss de 50% pendant 1 tour.</t>
+        </is>
+      </c>
+      <c r="P3" s="173" t="inlineStr">
+        <is>
+          <t>« Le froid n'est pas une punition, c'est une vérité. »</t>
+        </is>
+      </c>
+      <c r="Q3" s="172" t="inlineStr">
+        <is>
+          <t>drop:corrupted_dryad</t>
+        </is>
+      </c>
+      <c r="R3" s="173" t="inlineStr">
+        <is>
+          <t>Drop rare de la Dryade Corrompue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="165" t="inlineStr">
+        <is>
+          <t>ifrit</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Ifrit</t>
+        </is>
+      </c>
+      <c r="C4" s="167" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
+      <c r="D4" s="168" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="E4" s="167" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F4" s="167" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G4" s="167" t="n">
+        <v>130</v>
+      </c>
+      <c r="H4" s="167" t="n"/>
+      <c r="I4" s="167" t="n"/>
+      <c r="J4" s="167" t="n"/>
+      <c r="K4" s="167" t="n"/>
+      <c r="L4" s="167" t="n"/>
+      <c r="M4" s="167" t="n"/>
+      <c r="N4" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="169" t="inlineStr">
+        <is>
+          <t>Dégâts de feu purs. Multiplicateur élémentaire appliqué si le boss a un élément.</t>
+        </is>
+      </c>
+      <c r="P4" s="169" t="inlineStr">
+        <is>
+          <t>« La flamme ne demande pas la permission. »</t>
+        </is>
+      </c>
+      <c r="Q4" s="167" t="inlineStr">
+        <is>
+          <t>drop:goblin_woods</t>
+        </is>
+      </c>
+      <c r="R4" s="169" t="inlineStr">
+        <is>
+          <t>Drop rare du Gobelin des Bois</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="170" t="inlineStr">
+        <is>
+          <t>ramuh</t>
+        </is>
+      </c>
+      <c r="B5" s="171" t="inlineStr">
+        <is>
+          <t>Ramuh</t>
+        </is>
+      </c>
+      <c r="C5" s="172" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="D5" s="174" t="inlineStr">
+        <is>
+          <t>Épique</t>
+        </is>
+      </c>
+      <c r="E5" s="172" t="inlineStr">
+        <is>
+          <t>lightning</t>
+        </is>
+      </c>
+      <c r="F5" s="172" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G5" s="172" t="n">
+        <v>180</v>
+      </c>
+      <c r="H5" s="172" t="n"/>
+      <c r="I5" s="172" t="n"/>
+      <c r="J5" s="172" t="n"/>
+      <c r="K5" s="172" t="inlineStr">
+        <is>
+          <t>boss_stun</t>
+        </is>
+      </c>
+      <c r="L5" s="172" t="inlineStr">
+        <is>
+          <t>turns:1</t>
+        </is>
+      </c>
+      <c r="M5" s="172" t="n"/>
+      <c r="N5" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="173" t="inlineStr">
+        <is>
+          <t>Frappe de foudre + étourdissement du boss (pas de contre-attaque ce tour).</t>
+        </is>
+      </c>
+      <c r="P5" s="173" t="inlineStr">
+        <is>
+          <t>« Le jugement tombe vite et sans appel. »</t>
+        </is>
+      </c>
+      <c r="Q5" s="172" t="inlineStr">
+        <is>
+          <t>drop:wolf_alpha</t>
+        </is>
+      </c>
+      <c r="R5" s="173" t="inlineStr">
+        <is>
+          <t>Drop rare du Loup Alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="165" t="inlineStr">
+        <is>
+          <t>leviathan</t>
+        </is>
+      </c>
+      <c r="B6" s="166" t="inlineStr">
+        <is>
+          <t>Léviathan</t>
+        </is>
+      </c>
+      <c r="C6" s="167" t="inlineStr">
+        <is>
+          <t>🌊</t>
+        </is>
+      </c>
+      <c r="D6" s="174" t="inlineStr">
+        <is>
+          <t>Épique</t>
+        </is>
+      </c>
+      <c r="E6" s="167" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="F6" s="167" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G6" s="167" t="n">
+        <v>150</v>
+      </c>
+      <c r="H6" s="167" t="n"/>
+      <c r="I6" s="167" t="n"/>
+      <c r="J6" s="167" t="n"/>
+      <c r="K6" s="167" t="inlineStr">
+        <is>
+          <t>heal_pct</t>
+        </is>
+      </c>
+      <c r="L6" s="167" t="inlineStr">
+        <is>
+          <t>value:0.3</t>
+        </is>
+      </c>
+      <c r="M6" s="167" t="n"/>
+      <c r="N6" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="169" t="inlineStr">
+        <is>
+          <t>150 dégâts + restaure 30% des PV max du joueur.</t>
+        </is>
+      </c>
+      <c r="P6" s="169" t="inlineStr">
+        <is>
+          <t>« L'eau donne et reprend à sa guise. »</t>
+        </is>
+      </c>
+      <c r="Q6" s="167" t="inlineStr">
+        <is>
+          <t>drop:swamp_troll</t>
+        </is>
+      </c>
+      <c r="R6" s="169" t="inlineStr">
+        <is>
+          <t>Drop rare du Troll des Marais</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="170" t="inlineStr">
+        <is>
+          <t>odin</t>
+        </is>
+      </c>
+      <c r="B7" s="171" t="inlineStr">
+        <is>
+          <t>Odin</t>
+        </is>
+      </c>
+      <c r="C7" s="172" t="inlineStr">
+        <is>
+          <t>☠️</t>
+        </is>
+      </c>
+      <c r="D7" s="174" t="inlineStr">
+        <is>
+          <t>Épique</t>
+        </is>
+      </c>
+      <c r="E7" s="172" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="F7" s="172" t="inlineStr">
+        <is>
+          <t>instakill_or_damage</t>
+        </is>
+      </c>
+      <c r="G7" s="172" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" s="172" t="n"/>
+      <c r="I7" s="172" t="n"/>
+      <c r="J7" s="172" t="n"/>
+      <c r="K7" s="172" t="n"/>
+      <c r="L7" s="172" t="n"/>
+      <c r="M7" s="172" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N7" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="173" t="inlineStr">
+        <is>
+          <t>Boss &lt; 30% PV → mort instantanée (Odinfell). Sinon 200 dégâts.</t>
+        </is>
+      </c>
+      <c r="P7" s="173" t="inlineStr">
+        <is>
+          <t>« Certains destins ne connaissent pas d'appel. »</t>
+        </is>
+      </c>
+      <c r="Q7" s="172" t="inlineStr">
+        <is>
+          <t>drop:witch_woods</t>
+        </is>
+      </c>
+      <c r="R7" s="173" t="inlineStr">
+        <is>
+          <t>Drop rare de la Sorcière des Bois</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="165" t="inlineStr">
+        <is>
+          <t>alexander</t>
+        </is>
+      </c>
+      <c r="B8" s="166" t="inlineStr">
+        <is>
+          <t>Alexander</t>
+        </is>
+      </c>
+      <c r="C8" s="167" t="inlineStr">
+        <is>
+          <t>🏰</t>
+        </is>
+      </c>
+      <c r="D8" s="174" t="inlineStr">
+        <is>
+          <t>Épique</t>
+        </is>
+      </c>
+      <c r="E8" s="167" t="inlineStr">
+        <is>
+          <t>holy</t>
+        </is>
+      </c>
+      <c r="F8" s="167" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G8" s="167" t="n">
+        <v>160</v>
+      </c>
+      <c r="H8" s="167" t="n"/>
+      <c r="I8" s="167" t="n"/>
+      <c r="J8" s="167" t="n"/>
+      <c r="K8" s="167" t="inlineStr">
+        <is>
+          <t>restore_mp</t>
+        </is>
+      </c>
+      <c r="L8" s="167" t="inlineStr">
+        <is>
+          <t>value:35</t>
+        </is>
+      </c>
+      <c r="M8" s="167" t="n"/>
+      <c r="N8" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="169" t="inlineStr">
+        <is>
+          <t>160 dégâts + restaure 35 MP au joueur.</t>
+        </is>
+      </c>
+      <c r="P8" s="169" t="inlineStr">
+        <is>
+          <t>« Le sacré protège autant qu'il détruit. »</t>
+        </is>
+      </c>
+      <c r="Q8" s="167" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="R8" s="169" t="inlineStr">
+        <is>
+          <t>Quête 'Lumière des Anciens' — vaincre 10 boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="170" t="inlineStr">
+        <is>
+          <t>bahamut</t>
+        </is>
+      </c>
+      <c r="B9" s="171" t="inlineStr">
+        <is>
+          <t>Bahamut</t>
+        </is>
+      </c>
+      <c r="C9" s="172" t="inlineStr">
+        <is>
+          <t>🐲</t>
+        </is>
+      </c>
+      <c r="D9" s="175" t="inlineStr">
+        <is>
+          <t>Légendaire</t>
+        </is>
+      </c>
+      <c r="E9" s="172" t="inlineStr">
+        <is>
+          <t>wind</t>
+        </is>
+      </c>
+      <c r="F9" s="172" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G9" s="172" t="n">
+        <v>350</v>
+      </c>
+      <c r="H9" s="172" t="n"/>
+      <c r="I9" s="172" t="n"/>
+      <c r="J9" s="172" t="n"/>
+      <c r="K9" s="172" t="n"/>
+      <c r="L9" s="172" t="n"/>
+      <c r="M9" s="172" t="n"/>
+      <c r="N9" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="173" t="inlineStr">
+        <is>
+          <t>Mégaflare : 350 dégâts purs. Aucun effet secondaire.</t>
+        </is>
+      </c>
+      <c r="P9" s="173" t="inlineStr">
+        <is>
+          <t>« Face au roi des dragons, l'orgueil se tait. »</t>
+        </is>
+      </c>
+      <c r="Q9" s="172" t="inlineStr">
+        <is>
+          <t>regional:wolf_king</t>
+        </is>
+      </c>
+      <c r="R9" s="173" t="inlineStr">
+        <is>
+          <t>Drop Boss Régional Roi des Loups</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="165" t="inlineStr">
+        <is>
+          <t>phoenix</t>
+        </is>
+      </c>
+      <c r="B10" s="166" t="inlineStr">
+        <is>
+          <t>Phénix</t>
+        </is>
+      </c>
+      <c r="C10" s="167" t="inlineStr">
+        <is>
+          <t>🦅</t>
+        </is>
+      </c>
+      <c r="D10" s="175" t="inlineStr">
+        <is>
+          <t>Légendaire</t>
+        </is>
+      </c>
+      <c r="E10" s="167" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F10" s="167" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="G10" s="167" t="n">
+        <v>220</v>
+      </c>
+      <c r="H10" s="167" t="n"/>
+      <c r="I10" s="167" t="n"/>
+      <c r="J10" s="167" t="n"/>
+      <c r="K10" s="167" t="inlineStr">
+        <is>
+          <t>conditional_heal</t>
+        </is>
+      </c>
+      <c r="L10" s="167" t="inlineStr">
+        <is>
+          <t>hpThreshold:0.4,healTo:0.65</t>
+        </is>
+      </c>
+      <c r="M10" s="167" t="n"/>
+      <c r="N10" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="169" t="inlineStr">
+        <is>
+          <t>220 dégâts. Si joueur &lt; 40% PV → soin à 65% PV max.</t>
+        </is>
+      </c>
+      <c r="P10" s="169" t="inlineStr">
+        <is>
+          <t>« De la cendre naît la force. »</t>
+        </is>
+      </c>
+      <c r="Q10" s="167" t="inlineStr">
+        <is>
+          <t>drop:cursed_fairy</t>
+        </is>
+      </c>
+      <c r="R10" s="169" t="inlineStr">
+        <is>
+          <t>Drop rare de la Fée Maudite</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="170" t="inlineStr">
+        <is>
+          <t>knights_of_round</t>
+        </is>
+      </c>
+      <c r="B11" s="171" t="inlineStr">
+        <is>
+          <t>Chevaliers de la Table</t>
+        </is>
+      </c>
+      <c r="C11" s="172" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="D11" s="175" t="inlineStr">
+        <is>
+          <t>Légendaire</t>
+        </is>
+      </c>
+      <c r="E11" s="172" t="n"/>
+      <c r="F11" s="172" t="inlineStr">
+        <is>
+          <t>multihit</t>
+        </is>
+      </c>
+      <c r="G11" s="172" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="172" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" s="172" t="n"/>
+      <c r="J11" s="172" t="n"/>
+      <c r="K11" s="172" t="n"/>
+      <c r="L11" s="172" t="n"/>
+      <c r="M11" s="172" t="n"/>
+      <c r="N11" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="173" t="inlineStr">
+        <is>
+          <t>5 frappes × 100 dégâts = 500 dégâts totaux.</t>
+        </is>
+      </c>
+      <c r="P11" s="173" t="inlineStr">
+        <is>
+          <t>« Seuls les plus vaillants méritent leur aide. »</t>
+        </is>
+      </c>
+      <c r="Q11" s="172" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="R11" s="173" t="inlineStr">
+        <is>
+          <t>Forge légendaire : 3× Fang d'Argent + 2× Cristal de Mana + 1× Os Runique</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="176" t="inlineStr">
+        <is>
+          <t>⚙️ MÉCANIQUE GÉNÉRALE</t>
+        </is>
+      </c>
+      <c r="B1" s="182" t="n"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="177" t="inlineStr">
+        <is>
+          <t>Emplacements max équipés</t>
+        </is>
+      </c>
+      <c r="B2" s="178" t="inlineStr">
+        <is>
+          <t>3 invocations différentes en simultané (choix dans l'inventaire Hub)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="179" t="inlineStr">
+        <is>
+          <t>Usages par combat</t>
+        </is>
+      </c>
+      <c r="B3" s="180" t="inlineStr">
+        <is>
+          <t>1 seul usage par invocation et par combat — impossible de répéter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="177" t="inlineStr">
+        <is>
+          <t>Jauge (Gauge)</t>
+        </is>
+      </c>
+      <c r="B4" s="178" t="inlineStr">
+        <is>
+          <t>Se remplit de +25% à chaque contre-attaque boss reçue. 4 coups = pleine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="179" t="inlineStr">
+        <is>
+          <t>Activation</t>
+        </is>
+      </c>
+      <c r="B5" s="180" t="inlineStr">
+        <is>
+          <t>Jauge à 100% requis. Se remet à 0 après chaque utilisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="177" t="inlineStr">
+        <is>
+          <t>Persistance</t>
+        </is>
+      </c>
+      <c r="B6" s="178" t="inlineStr">
+        <is>
+          <t>La jauge repart à 0 entre les combats. Ne persiste PAS entre les séances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="179" t="inlineStr">
+        <is>
+          <t>Cumul avec Limite</t>
+        </is>
+      </c>
+      <c r="B7" s="180" t="inlineStr">
+        <is>
+          <t>La jauge d'invocation se remplit EN PARALLÈLE de la barre de Limite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="176" t="inlineStr">
+        <is>
+          <t>⚡ EFFETS PRINCIPAUX</t>
+        </is>
+      </c>
+      <c r="B8" s="182" t="n"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="179" t="inlineStr">
+        <is>
+          <t>damage_force</t>
+        </is>
+      </c>
+      <c r="B9" s="180" t="inlineStr">
+        <is>
+          <t>Dégâts = baseDamage + force_joueur × stat_scale_mult (Titan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="177" t="inlineStr">
+        <is>
+          <t>damage_flat</t>
+        </is>
+      </c>
+      <c r="B10" s="178" t="inlineStr">
+        <is>
+          <t>Dégâts fixes (avec multiplicateur élémentaire si applicable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="179" t="inlineStr">
+        <is>
+          <t>instakill_or_damage</t>
+        </is>
+      </c>
+      <c r="B11" s="180" t="inlineStr">
+        <is>
+          <t>Boss &lt; instakill_thresh PV → mort immédiate. Sinon → dégâts normaux. (Odin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="177" t="inlineStr">
+        <is>
+          <t>multihit</t>
+        </is>
+      </c>
+      <c r="B12" s="178" t="inlineStr">
+        <is>
+          <t>N frappes × base_damage_per_hit. Total = hits × base_damage. (Chevaliers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="176" t="inlineStr">
+        <is>
+          <t>✨ EFFETS SECONDAIRES</t>
+        </is>
+      </c>
+      <c r="B13" s="182" t="n"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="177" t="inlineStr">
+        <is>
+          <t>boss_weaken</t>
+        </is>
+      </c>
+      <c r="B14" s="178" t="inlineStr">
+        <is>
+          <t>Réduit les dégâts de la prochaine contre-attaque boss (réduction en %). Dure N tours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="179" t="inlineStr">
+        <is>
+          <t>boss_stun</t>
+        </is>
+      </c>
+      <c r="B15" s="180" t="inlineStr">
+        <is>
+          <t>Le boss saute sa contre-attaque ce tour. Dure N tours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="177" t="inlineStr">
+        <is>
+          <t>heal_pct</t>
+        </is>
+      </c>
+      <c r="B16" s="178" t="inlineStr">
+        <is>
+          <t>Restaure X% des PV MAX du joueur (indépendant des PV actuels).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="179" t="inlineStr">
+        <is>
+          <t>restore_mp</t>
+        </is>
+      </c>
+      <c r="B17" s="180" t="inlineStr">
+        <is>
+          <t>Restaure X MP au joueur instantanément.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="177" t="inlineStr">
+        <is>
+          <t>conditional_heal</t>
+        </is>
+      </c>
+      <c r="B18" s="178" t="inlineStr">
+        <is>
+          <t>Soin à healTo % PV uniquement si joueur &lt; hpThreshold % PV. Sinon aucun soin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="176" t="inlineStr">
+        <is>
+          <t>📍 OBTENTION</t>
+        </is>
+      </c>
+      <c r="B19" s="182" t="n"/>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="177" t="inlineStr">
+        <is>
+          <t>drop:&lt;boss_id&gt;</t>
+        </is>
+      </c>
+      <c r="B20" s="178" t="inlineStr">
+        <is>
+          <t>Drop rare aléatoire à chaque victoire sur le boss indiqué.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="179" t="inlineStr">
+        <is>
+          <t>regional:&lt;boss_id&gt;</t>
+        </is>
+      </c>
+      <c r="B21" s="180" t="inlineStr">
+        <is>
+          <t>Drop du boss régional de zone (boss de fin de zone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="177" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="B22" s="178" t="inlineStr">
+        <is>
+          <t>Récompense de quête spéciale (Alexander : vaincre 10 boss différents).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="179" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="B23" s="180" t="inlineStr">
+        <is>
+          <t>Recette légendaire au Forgeron (matériaux rares requis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="177" t="inlineStr">
+        <is>
+          <t>Admin → Invocations</t>
+        </is>
+      </c>
+      <c r="B24" s="178" t="inlineStr">
+        <is>
+          <t>L'administrateur peut donner/retirer des invocations depuis le panneau admin.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14968,7 +16255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:W16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14989,6 +16276,8 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="35" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="21" max="21"/>
+    <col width="60" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -15012,6 +16301,11 @@
           <t>📝 INFO</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>🎞 MÉDIAS</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="147" t="inlineStr">
@@ -15133,7 +16427,19 @@
 affichée</t>
         </is>
       </c>
-      <c r="U2" s="126" t="inlineStr">
+      <c r="U2" s="181" t="inlineStr">
+        <is>
+          <t>Miniature
+(thumbUrl Giphy 200px)</t>
+        </is>
+      </c>
+      <c r="V2" s="181" t="inlineStr">
+        <is>
+          <t>GIF animé
+(gifUrl Giphy full)</t>
+        </is>
+      </c>
+      <c r="W2" s="126" t="inlineStr">
         <is>
           <t>Notes Game
 Design</t>
@@ -15216,10 +16522,20 @@
       </c>
       <c r="T3" s="141" t="inlineStr">
         <is>
-          <t>Effectue des pompes complètes au sol.</t>
-        </is>
-      </c>
-      <c r="U3" s="141" t="inlineStr">
+          <t>Effectue des pompes complètes au sol, bras à largeur d'épaules. Descends jusqu'à ce que la poitrine frôle le sol, puis remonte en gardant le corps bien droit.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/3ohze1qkqPZHMrEuwo/200.gif</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/3ohze1qkqPZHMrEuwo/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W3" s="141" t="inlineStr">
         <is>
           <t>Exercice de base, force haut du corps.</t>
         </is>
@@ -15301,10 +16617,20 @@
       </c>
       <c r="T4" s="141" t="inlineStr">
         <is>
-          <t>Descends jusqu'à ce que les cuisses soient parallèles au sol.</t>
-        </is>
-      </c>
-      <c r="U4" s="141" t="inlineStr">
+          <t>Descends jusqu'à ce que les cuisses soient parallèles au sol, dos droit et talons à plat. Pousse sur les talons pour remonter.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/tHyPJtOwPChKmF0LKg/200.gif</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/tHyPJtOwPChKmF0LKg/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W4" s="141" t="inlineStr">
         <is>
           <t>Exercice majeur bas du corps.</t>
         </is>
@@ -15386,10 +16712,20 @@
       </c>
       <c r="T5" s="152" t="inlineStr">
         <is>
-          <t>Maintiens la position de gainage les bras tendus.</t>
-        </is>
-      </c>
-      <c r="U5" s="152" t="inlineStr">
+          <t>Maintiens la position de gainage les bras tendus, corps aligné de la tête aux pieds. Contracte les abdos et respire régulièrement.</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/ZcteOOkovIh9HaVFjT/200.gif</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/ZcteOOkovIh9HaVFjT/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W5" s="152" t="inlineStr">
         <is>
           <t>Exercice isométrique, renforce le centre.</t>
         </is>
@@ -15471,10 +16807,20 @@
       </c>
       <c r="T6" s="133" t="inlineStr">
         <is>
-          <t>Pompe + saut vertical, le tout enchaîné.</t>
-        </is>
-      </c>
-      <c r="U6" s="133" t="inlineStr">
+          <t>Debout, accroupis, place les mains au sol, saute en position de pompe, reviens accroupi puis saute verticalement en levant les bras.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/KxuGSIZU1QZfRiRx4h/200.gif</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/KxuGSIZU1QZfRiRx4h/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W6" s="133" t="inlineStr">
         <is>
           <t>Exercice à haute intensité, excellent pour le cardio.</t>
         </is>
@@ -15556,10 +16902,20 @@
       </c>
       <c r="T7" s="133" t="inlineStr">
         <is>
-          <t>Sauts en écartant les bras et jambes en même temps.</t>
-        </is>
-      </c>
-      <c r="U7" s="133" t="inlineStr">
+          <t>Saute en écartant simultanément les bras et les jambes, puis reviens en position initiale. Maintiens un rythme régulier.</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>https://media0.giphy.com/media/RgtuKqJ8rPII4qdRjp/200.gif</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>https://media0.giphy.com/media/RgtuKqJ8rPII4qdRjp/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W7" s="133" t="inlineStr">
         <is>
           <t>Exercice cardio léger, parfait pour l'échauffement.</t>
         </is>
@@ -15641,10 +16997,20 @@
       </c>
       <c r="T8" s="141" t="inlineStr">
         <is>
-          <t>Alterne les fentes avant gauche/droite.</t>
-        </is>
-      </c>
-      <c r="U8" s="141" t="inlineStr">
+          <t>Alterne les fentes avant gauche/droite. Le genou avant ne doit pas dépasser le bout du pied, le genou arrière effleure le sol.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>https://media0.giphy.com/media/BDta60HEH7374d4lSZ/200.gif</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>https://media0.giphy.com/media/BDta60HEH7374d4lSZ/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W8" s="141" t="inlineStr">
         <is>
           <t>Renforce quadriceps et fessiers.</t>
         </is>
@@ -15726,10 +17092,20 @@
       </c>
       <c r="T9" s="133" t="inlineStr">
         <is>
-          <t>Cours sur place en levant bien les genoux.</t>
-        </is>
-      </c>
-      <c r="U9" s="133" t="inlineStr">
+          <t>Cours sur place en levant bien les genoux à hauteur de la hanche. Bras fléchis à 90°, mouvement naturel de la course.</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/VpDGbWPepQNWDFO0Jo/200.gif</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/VpDGbWPepQNWDFO0Jo/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W9" s="133" t="inlineStr">
         <is>
           <t>Cardio sans déplacement, augmente l'endurance.</t>
         </is>
@@ -15811,10 +17187,20 @@
       </c>
       <c r="T10" s="141" t="inlineStr">
         <is>
-          <t>Dips sur le bord d'une chaise, bras en arrière.</t>
-        </is>
-      </c>
-      <c r="U10" s="141" t="inlineStr">
+          <t>Assis sur le bord d'une chaise, mains de chaque côté des hanches. Glisse vers l'avant et descends en fléchissant les coudes à 90°, puis remonte.</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/4zIMiq61O8M2ZBxfRv/200.gif</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/4zIMiq61O8M2ZBxfRv/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W10" s="141" t="inlineStr">
         <is>
           <t>Renforce les triceps. Équipement simple.</t>
         </is>
@@ -15896,10 +17282,20 @@
       </c>
       <c r="T11" s="133" t="inlineStr">
         <is>
-          <t>En position de pompe, ramène les genoux vers la poitrine en alternance.</t>
-        </is>
-      </c>
-      <c r="U11" s="133" t="inlineStr">
+          <t>En position de pompe, ramène les genoux vers la poitrine en alternance le plus vite possible. Garde les hanches basses.</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/VzlPEkuoqlgjehxvxk/200.gif</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>https://media1.giphy.com/media/VzlPEkuoqlgjehxvxk/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W11" s="133" t="inlineStr">
         <is>
           <t>Cardio + gainage combinés.</t>
         </is>
@@ -15981,10 +17377,20 @@
       </c>
       <c r="T12" s="152" t="inlineStr">
         <is>
-          <t>Dos contre le mur, cuisses à 90° pendant toute la durée.</t>
-        </is>
-      </c>
-      <c r="U12" s="152" t="inlineStr">
+          <t>Dos contre le mur, cuisses à 90° et pieds à plat au sol. Maintiens la position pendant toute la durée, bras tendus le long du corps.</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/wiRXDJkS5rcMQ2oSJG/200.gif</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/wiRXDJkS5rcMQ2oSJG/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W12" s="152" t="inlineStr">
         <is>
           <t>Exercice isométrique, endurance des jambes.</t>
         </is>
@@ -16066,10 +17472,20 @@
       </c>
       <c r="T13" s="133" t="inlineStr">
         <is>
-          <t>Lève les genoux le plus haut possible en alternance.</t>
-        </is>
-      </c>
-      <c r="U13" s="133" t="inlineStr">
+          <t>Lève les genoux le plus haut possible en alternance, idéalement à hauteur de hanche. Bras qui accompagnent le mouvement.</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/l0HlNOsSRC0Bts7iU/200.gif</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>https://media3.giphy.com/media/l0HlNOsSRC0Bts7iU/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W13" s="133" t="inlineStr">
         <is>
           <t>Cardio et coordination.</t>
         </is>
@@ -16151,15 +17567,26 @@
       </c>
       <c r="T14" s="141" t="inlineStr">
         <is>
-          <t>Soulève les épaules du sol, contracte les abdos.</t>
-        </is>
-      </c>
-      <c r="U14" s="141" t="inlineStr">
+          <t>Allongé sur le dos, genoux fléchis, mains derrière la tête. Soulève les épaules du sol en contractant les abdos, sans tirer sur la nuque.</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/OgJiGwuIlVvgs/200.gif</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>https://media2.giphy.com/media/OgJiGwuIlVvgs/giphy.gif</t>
+        </is>
+      </c>
+      <c r="W14" s="141" t="inlineStr">
         <is>
           <t>Renforce les abdominaux.</t>
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="153" t="inlineStr">
         <is>

</xml_diff>